<commit_message>
chore: quarterly retrain (2026-06-27)
</commit_message>
<xml_diff>
--- a/wsts_historical.xlsx
+++ b/wsts_historical.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tpwsts-my.sharepoint.com/personal/admin_tpwsts_onmicrosoft_com/Documents/WSTS/2-WSTS-Statistic-Reports/Blue Book/Blue Book 2026/BB-01-26/BB-01-26-final/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tpwsts-my.sharepoint.com/personal/admin_tpwsts_onmicrosoft_com/Documents/WSTS/2-WSTS-Statistic-Reports/Blue Book/Blue Book 2026/BB-04-26/BB-04-26-final/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="36" documentId="13_ncr:1_{95B6A9BD-11A5-4993-BD56-443C8CBE0F5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1EB4657E-16F0-4995-A4BE-8FC74933C6FE}"/>
+  <xr:revisionPtr revIDLastSave="45" documentId="13_ncr:1_{95B6A9BD-11A5-4993-BD56-443C8CBE0F5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D9A45AF1-3CE6-4FBB-8E4C-CA54551C8938}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="24220" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Monthly Data" sheetId="1" r:id="rId1"/>
@@ -244,53 +244,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{BDC5686E-BE8A-4354-A574-F80CBEE9F63A}"/>
   </cellStyles>
-  <dxfs count="22">
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor indexed="43"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor indexed="43"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="18">
     <dxf>
       <border>
         <left style="thin">
@@ -603,7 +557,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>581025</xdr:colOff>
+      <xdr:colOff>581024</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
@@ -959,19 +913,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:R250"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.75" style="7" customWidth="1"/>
-    <col min="2" max="2" width="10.375" customWidth="1"/>
-    <col min="3" max="9" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="10.375" customWidth="1"/>
-    <col min="14" max="14" width="11.5" style="7" customWidth="1"/>
-    <col min="15" max="18" width="11.125" style="10" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.77734375" style="7" customWidth="1"/>
+    <col min="2" max="2" width="10.33203125" customWidth="1"/>
+    <col min="3" max="9" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="10.33203125" customWidth="1"/>
+    <col min="14" max="14" width="11.44140625" style="7" customWidth="1"/>
+    <col min="15" max="18" width="11.109375" style="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" ht="18" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>26</v>
       </c>
@@ -979,7 +933,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" ht="18" x14ac:dyDescent="0.4">
       <c r="A2" s="3" t="s">
         <v>27</v>
       </c>
@@ -14328,11 +14282,17 @@
         <v>1</v>
       </c>
       <c r="B246" s="6">
-        <v>24507492</v>
-      </c>
-      <c r="C246" s="6"/>
-      <c r="D246" s="6"/>
-      <c r="E246" s="6"/>
+        <v>24625051</v>
+      </c>
+      <c r="C246" s="6">
+        <v>36199755</v>
+      </c>
+      <c r="D246" s="6">
+        <v>40595854</v>
+      </c>
+      <c r="E246" s="6">
+        <v>41534424</v>
+      </c>
       <c r="F246" s="6"/>
       <c r="G246" s="6"/>
       <c r="H246" s="6"/>
@@ -14343,15 +14303,15 @@
       <c r="M246" s="5"/>
       <c r="N246" s="8">
         <f>SUM(B246:M246)</f>
-        <v>24507492</v>
+        <v>142955084</v>
       </c>
       <c r="O246" s="11">
         <f>SUM(B246:D246)</f>
-        <v>24507492</v>
+        <v>101420660</v>
       </c>
       <c r="P246" s="11">
         <f>SUM(E246:G246)</f>
-        <v>0</v>
+        <v>41534424</v>
       </c>
       <c r="Q246" s="11">
         <f>SUM(H246:J246)</f>
@@ -14367,11 +14327,17 @@
         <v>2</v>
       </c>
       <c r="B247" s="6">
-        <v>5493060</v>
-      </c>
-      <c r="C247" s="6"/>
-      <c r="D247" s="6"/>
-      <c r="E247" s="6"/>
+        <v>5506393</v>
+      </c>
+      <c r="C247" s="6">
+        <v>6560532</v>
+      </c>
+      <c r="D247" s="6">
+        <v>6530959</v>
+      </c>
+      <c r="E247" s="6">
+        <v>6754705</v>
+      </c>
       <c r="F247" s="6"/>
       <c r="G247" s="6"/>
       <c r="H247" s="6"/>
@@ -14382,15 +14348,15 @@
       <c r="M247" s="5"/>
       <c r="N247" s="8">
         <f>SUM(B247:M247)</f>
-        <v>5493060</v>
+        <v>25352589</v>
       </c>
       <c r="O247" s="11">
         <f>SUM(B247:D247)</f>
-        <v>5493060</v>
+        <v>18597884</v>
       </c>
       <c r="P247" s="11">
         <f>SUM(E247:G247)</f>
-        <v>0</v>
+        <v>6754705</v>
       </c>
       <c r="Q247" s="11">
         <f>SUM(H247:J247)</f>
@@ -14406,11 +14372,17 @@
         <v>3</v>
       </c>
       <c r="B248" s="6">
-        <v>3641116</v>
-      </c>
-      <c r="C248" s="6"/>
-      <c r="D248" s="6"/>
-      <c r="E248" s="6"/>
+        <v>3650632</v>
+      </c>
+      <c r="C248" s="6">
+        <v>4032095</v>
+      </c>
+      <c r="D248" s="6">
+        <v>4467292</v>
+      </c>
+      <c r="E248" s="6">
+        <v>4428604</v>
+      </c>
       <c r="F248" s="6"/>
       <c r="G248" s="6"/>
       <c r="H248" s="6"/>
@@ -14421,15 +14393,15 @@
       <c r="M248" s="5"/>
       <c r="N248" s="8">
         <f>SUM(B248:M248)</f>
-        <v>3641116</v>
+        <v>16578623</v>
       </c>
       <c r="O248" s="11">
         <f>SUM(B248:D248)</f>
-        <v>3641116</v>
+        <v>12150019</v>
       </c>
       <c r="P248" s="11">
         <f>SUM(E248:G248)</f>
-        <v>0</v>
+        <v>4428604</v>
       </c>
       <c r="Q248" s="11">
         <f>SUM(H248:J248)</f>
@@ -14445,11 +14417,17 @@
         <v>4</v>
       </c>
       <c r="B249" s="6">
-        <v>46742805</v>
-      </c>
-      <c r="C249" s="6"/>
-      <c r="D249" s="6"/>
-      <c r="E249" s="6"/>
+        <v>46998751</v>
+      </c>
+      <c r="C249" s="6">
+        <v>54762826</v>
+      </c>
+      <c r="D249" s="6">
+        <v>64615492</v>
+      </c>
+      <c r="E249" s="6">
+        <v>60958983</v>
+      </c>
       <c r="F249" s="6"/>
       <c r="G249" s="6"/>
       <c r="H249" s="6"/>
@@ -14460,15 +14438,15 @@
       <c r="M249" s="5"/>
       <c r="N249" s="8">
         <f>SUM(B249:M249)</f>
-        <v>46742805</v>
+        <v>227336052</v>
       </c>
       <c r="O249" s="11">
         <f>SUM(B249:D249)</f>
-        <v>46742805</v>
+        <v>166377069</v>
       </c>
       <c r="P249" s="11">
         <f>SUM(E249:G249)</f>
-        <v>0</v>
+        <v>60958983</v>
       </c>
       <c r="Q249" s="11">
         <f>SUM(H249:J249)</f>
@@ -14484,11 +14462,17 @@
         <v>0</v>
       </c>
       <c r="B250" s="6">
-        <v>80384473</v>
-      </c>
-      <c r="C250" s="6"/>
-      <c r="D250" s="6"/>
-      <c r="E250" s="6"/>
+        <v>80780827</v>
+      </c>
+      <c r="C250" s="6">
+        <v>101555208</v>
+      </c>
+      <c r="D250" s="6">
+        <v>116209597</v>
+      </c>
+      <c r="E250" s="6">
+        <v>113676716</v>
+      </c>
       <c r="F250" s="6"/>
       <c r="G250" s="6"/>
       <c r="H250" s="6"/>
@@ -14499,15 +14483,15 @@
       <c r="M250" s="5"/>
       <c r="N250" s="8">
         <f>SUM(N246:N249)</f>
-        <v>80384473</v>
+        <v>412222348</v>
       </c>
       <c r="O250" s="11">
         <f>SUM(B250:D250)</f>
-        <v>80384473</v>
+        <v>298545632</v>
       </c>
       <c r="P250" s="11">
         <f>SUM(E250:G250)</f>
-        <v>0</v>
+        <v>113676716</v>
       </c>
       <c r="Q250" s="11">
         <f>SUM(H250:J250)</f>
@@ -14521,79 +14505,71 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="A228:B230 B228:L232">
-    <cfRule type="expression" dxfId="21" priority="36" stopIfTrue="1">
+    <cfRule type="expression" dxfId="17" priority="36" stopIfTrue="1">
       <formula>ISTEXT($A228)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A228:B230">
-    <cfRule type="expression" dxfId="20" priority="35" stopIfTrue="1">
+    <cfRule type="expression" dxfId="16" priority="35" stopIfTrue="1">
       <formula>ISNUMBER($A228)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A231:K232">
-    <cfRule type="expression" dxfId="19" priority="43" stopIfTrue="1">
+    <cfRule type="expression" dxfId="15" priority="43" stopIfTrue="1">
       <formula>ISNUMBER($A231)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="44" stopIfTrue="1">
+    <cfRule type="expression" dxfId="14" priority="44" stopIfTrue="1">
       <formula>ISTEXT($A231)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5:R227">
-    <cfRule type="expression" dxfId="17" priority="49" stopIfTrue="1">
+    <cfRule type="expression" dxfId="13" priority="49" stopIfTrue="1">
       <formula>ISNUMBER($A5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="16" priority="50" stopIfTrue="1">
+    <cfRule type="expression" dxfId="12" priority="50" stopIfTrue="1">
       <formula>ISTEXT($A5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A233:R244">
-    <cfRule type="expression" dxfId="15" priority="5" stopIfTrue="1">
+  <conditionalFormatting sqref="A233:R250">
+    <cfRule type="expression" dxfId="11" priority="1" stopIfTrue="1">
       <formula>ISNUMBER($A233)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="14" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="10" priority="2" stopIfTrue="1">
       <formula>ISTEXT($A233)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B237:K238">
-    <cfRule type="expression" dxfId="13" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="9" priority="11" stopIfTrue="1">
       <formula>ISNUMBER($A237)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="12" stopIfTrue="1">
+    <cfRule type="expression" dxfId="8" priority="12" stopIfTrue="1">
       <formula>ISTEXT($A237)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B243:K244">
-    <cfRule type="expression" dxfId="11" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="7" priority="7" stopIfTrue="1">
       <formula>ISNUMBER($A243)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="8" stopIfTrue="1">
+    <cfRule type="expression" dxfId="6" priority="8" stopIfTrue="1">
       <formula>ISTEXT($A243)</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="B249:K250">
+    <cfRule type="expression" dxfId="5" priority="3" stopIfTrue="1">
+      <formula>ISNUMBER($A249)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="4" priority="4" stopIfTrue="1">
+      <formula>ISTEXT($A249)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B228:R232">
-    <cfRule type="expression" dxfId="9" priority="31" stopIfTrue="1">
+    <cfRule type="expression" dxfId="3" priority="31" stopIfTrue="1">
       <formula>ISNUMBER($A228)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M228:R232">
-    <cfRule type="expression" dxfId="8" priority="32" stopIfTrue="1">
+    <cfRule type="expression" dxfId="2" priority="32" stopIfTrue="1">
       <formula>ISTEXT($A228)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A245:R250">
-    <cfRule type="expression" dxfId="5" priority="1" stopIfTrue="1">
-      <formula>ISNUMBER($A245)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="4" priority="2" stopIfTrue="1">
-      <formula>ISTEXT($A245)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B249:K250">
-    <cfRule type="expression" dxfId="3" priority="3" stopIfTrue="1">
-      <formula>ISNUMBER($A249)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="2" priority="4" stopIfTrue="1">
-      <formula>ISTEXT($A249)</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions verticalCentered="1"/>
@@ -14610,16 +14586,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:M250"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.375" customWidth="1"/>
-    <col min="2" max="13" width="10.375" customWidth="1"/>
-    <col min="14" max="17" width="9.375" customWidth="1"/>
-    <col min="18" max="18" width="3.75" customWidth="1"/>
-    <col min="19" max="19" width="5.125" customWidth="1"/>
+    <col min="1" max="1" width="18.33203125" customWidth="1"/>
+    <col min="2" max="4" width="10.33203125" customWidth="1"/>
+    <col min="5" max="5" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="13" width="10.33203125" customWidth="1"/>
+    <col min="14" max="17" width="9.33203125" customWidth="1"/>
+    <col min="18" max="18" width="3.77734375" customWidth="1"/>
+    <col min="19" max="19" width="5.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="18" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>26</v>
       </c>
@@ -14627,14 +14605,14 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" ht="18" x14ac:dyDescent="0.4">
       <c r="A2" s="3" t="s">
         <v>27</v>
       </c>
       <c r="F2" s="1"/>
       <c r="M2" s="2"/>
     </row>
-    <row r="3" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -24724,19 +24702,19 @@
       </c>
       <c r="B246" s="5">
         <f>IF('Monthly Data'!B246=0,0,AVERAGE('Monthly Data'!L240,'Monthly Data'!M240,'Monthly Data'!B246))</f>
-        <v>26379456.333333332</v>
+        <v>26418642.666666668</v>
       </c>
       <c r="C246" s="6">
         <f>IF('Monthly Data'!C246=0,0,AVERAGE('Monthly Data'!M240,'Monthly Data'!B246,'Monthly Data'!C246))</f>
-        <v>0</v>
+        <v>29839642.333333332</v>
       </c>
       <c r="D246" s="5">
         <f>IF('Monthly Data'!D246=0,0,AVERAGE('Monthly Data'!B246,'Monthly Data'!C246,'Monthly Data'!D246))</f>
-        <v>0</v>
+        <v>33806886.666666664</v>
       </c>
       <c r="E246" s="5">
         <f>IF('Monthly Data'!E246=0,0,AVERAGE('Monthly Data'!C246,'Monthly Data'!D246,'Monthly Data'!E246))</f>
-        <v>0</v>
+        <v>39443344.333333336</v>
       </c>
       <c r="F246" s="5">
         <f>IF('Monthly Data'!F246=0,0,AVERAGE('Monthly Data'!D246,'Monthly Data'!E246,'Monthly Data'!F246))</f>
@@ -24777,19 +24755,19 @@
       </c>
       <c r="B247" s="5">
         <f>IF('Monthly Data'!B247=0,0,AVERAGE('Monthly Data'!L241,'Monthly Data'!M241,'Monthly Data'!B247))</f>
-        <v>5176571</v>
+        <v>5181015.333333333</v>
       </c>
       <c r="C247" s="6">
         <f>IF('Monthly Data'!C247=0,0,AVERAGE('Monthly Data'!M241,'Monthly Data'!B247,'Monthly Data'!C247))</f>
-        <v>0</v>
+        <v>5720586.333333333</v>
       </c>
       <c r="D247" s="5">
         <f>IF('Monthly Data'!D247=0,0,AVERAGE('Monthly Data'!B247,'Monthly Data'!C247,'Monthly Data'!D247))</f>
-        <v>0</v>
+        <v>6199294.666666667</v>
       </c>
       <c r="E247" s="5">
         <f>IF('Monthly Data'!E247=0,0,AVERAGE('Monthly Data'!C247,'Monthly Data'!D247,'Monthly Data'!E247))</f>
-        <v>0</v>
+        <v>6615398.666666667</v>
       </c>
       <c r="F247" s="5">
         <f>IF('Monthly Data'!F247=0,0,AVERAGE('Monthly Data'!D247,'Monthly Data'!E247,'Monthly Data'!F247))</f>
@@ -24830,19 +24808,19 @@
       </c>
       <c r="B248" s="5">
         <f>IF('Monthly Data'!B248=0,0,AVERAGE('Monthly Data'!L242,'Monthly Data'!M242,'Monthly Data'!B248))</f>
-        <v>3662994</v>
+        <v>3666166</v>
       </c>
       <c r="C248" s="6">
         <f>IF('Monthly Data'!C248=0,0,AVERAGE('Monthly Data'!M242,'Monthly Data'!B248,'Monthly Data'!C248))</f>
-        <v>0</v>
+        <v>3780755.6666666665</v>
       </c>
       <c r="D248" s="5">
         <f>IF('Monthly Data'!D248=0,0,AVERAGE('Monthly Data'!B248,'Monthly Data'!C248,'Monthly Data'!D248))</f>
-        <v>0</v>
+        <v>4050006.3333333335</v>
       </c>
       <c r="E248" s="5">
         <f>IF('Monthly Data'!E248=0,0,AVERAGE('Monthly Data'!C248,'Monthly Data'!D248,'Monthly Data'!E248))</f>
-        <v>0</v>
+        <v>4309330.333333333</v>
       </c>
       <c r="F248" s="5">
         <f>IF('Monthly Data'!F248=0,0,AVERAGE('Monthly Data'!D248,'Monthly Data'!E248,'Monthly Data'!F248))</f>
@@ -24883,19 +24861,19 @@
       </c>
       <c r="B249" s="5">
         <f>IF('Monthly Data'!B249=0,0,AVERAGE('Monthly Data'!L243,'Monthly Data'!M243,'Monthly Data'!B249))</f>
-        <v>47319570.333333336</v>
+        <v>47404885.666666664</v>
       </c>
       <c r="C249" s="6">
         <f>IF('Monthly Data'!C249=0,0,AVERAGE('Monthly Data'!M243,'Monthly Data'!B249,'Monthly Data'!C249))</f>
-        <v>0</v>
+        <v>49887119.666666664</v>
       </c>
       <c r="D249" s="5">
         <f>IF('Monthly Data'!D249=0,0,AVERAGE('Monthly Data'!B249,'Monthly Data'!C249,'Monthly Data'!D249))</f>
-        <v>0</v>
+        <v>55459023</v>
       </c>
       <c r="E249" s="5">
         <f>IF('Monthly Data'!E249=0,0,AVERAGE('Monthly Data'!C249,'Monthly Data'!D249,'Monthly Data'!E249))</f>
-        <v>0</v>
+        <v>60112433.666666664</v>
       </c>
       <c r="F249" s="5">
         <f>IF('Monthly Data'!F249=0,0,AVERAGE('Monthly Data'!D249,'Monthly Data'!E249,'Monthly Data'!F249))</f>
@@ -24936,19 +24914,19 @@
       </c>
       <c r="B250" s="5">
         <f>IF('Monthly Data'!B250=0,0,AVERAGE('Monthly Data'!L244,'Monthly Data'!M244,'Monthly Data'!B250))</f>
-        <v>82538591.666666672</v>
+        <v>82670709.666666672</v>
       </c>
       <c r="C250" s="5">
         <f>IF('Monthly Data'!C250=0,0,AVERAGE('Monthly Data'!M244,'Monthly Data'!B250,'Monthly Data'!C250))</f>
-        <v>0</v>
+        <v>89228104</v>
       </c>
       <c r="D250" s="5">
         <f>IF('Monthly Data'!D250=0,0,AVERAGE('Monthly Data'!B250,'Monthly Data'!C250,'Monthly Data'!D250))</f>
-        <v>0</v>
+        <v>99515210.666666672</v>
       </c>
       <c r="E250" s="5">
         <f>IF('Monthly Data'!E250=0,0,AVERAGE('Monthly Data'!C250,'Monthly Data'!D250,'Monthly Data'!E250))</f>
-        <v>0</v>
+        <v>110480507</v>
       </c>
       <c r="F250" s="5">
         <f>IF('Monthly Data'!F250=0,0,AVERAGE('Monthly Data'!D250,'Monthly Data'!E250,'Monthly Data'!F250))</f>
@@ -24985,20 +24963,12 @@
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="A5:M244">
-    <cfRule type="expression" dxfId="7" priority="3" stopIfTrue="1">
+  <conditionalFormatting sqref="A5:M250">
+    <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
       <formula>ISNUMBER($A5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="4" stopIfTrue="1">
+    <cfRule type="expression" dxfId="0" priority="2" stopIfTrue="1">
       <formula>ISTEXT($A5)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A245:M250">
-    <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
-      <formula>ISNUMBER($A245)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="0" priority="2" stopIfTrue="1">
-      <formula>ISTEXT($A245)</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>

</xml_diff>